<commit_message>
correct kittle trade and new pick trade
</commit_message>
<xml_diff>
--- a/OffSeason.xlsx
+++ b/OffSeason.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="621">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="624">
   <si>
     <t xml:space="preserve">No Chubb – John Olson</t>
   </si>
@@ -464,6 +464,9 @@
     <t xml:space="preserve">Isaiah Likely</t>
   </si>
   <si>
+    <t xml:space="preserve">Pat Freiermuth</t>
+  </si>
+  <si>
     <t xml:space="preserve">Myles Garrett</t>
   </si>
   <si>
@@ -479,7 +482,7 @@
     <t xml:space="preserve">Tucker Kraft</t>
   </si>
   <si>
-    <t xml:space="preserve">Pat Freiermuth</t>
+    <t xml:space="preserve">Cade Otten</t>
   </si>
   <si>
     <t xml:space="preserve">Nick bosa</t>
@@ -497,7 +500,7 @@
     <t xml:space="preserve">Erick all Jr</t>
   </si>
   <si>
-    <t xml:space="preserve">Cade Otten</t>
+    <t xml:space="preserve">Michael Mayer</t>
   </si>
   <si>
     <t xml:space="preserve">Maxxx Crosby</t>
@@ -515,7 +518,7 @@
     <t xml:space="preserve">Jessie Bates III</t>
   </si>
   <si>
-    <t xml:space="preserve">Michael Mayer</t>
+    <t xml:space="preserve">Brian Branch</t>
   </si>
   <si>
     <t xml:space="preserve">Will Anderson</t>
@@ -533,7 +536,7 @@
     <t xml:space="preserve">Xavier Woods</t>
   </si>
   <si>
-    <t xml:space="preserve">Brian Branch</t>
+    <t xml:space="preserve">Tre’von Moehrig</t>
   </si>
   <si>
     <t xml:space="preserve">LB</t>
@@ -554,7 +557,7 @@
     <t xml:space="preserve">Alontea Taylor</t>
   </si>
   <si>
-    <t xml:space="preserve">Tre’von Moehrig</t>
+    <t xml:space="preserve">Damar Hamlin</t>
   </si>
   <si>
     <t xml:space="preserve">Roquan Smith</t>
@@ -572,7 +575,7 @@
     <t xml:space="preserve">Devon Witherspoon</t>
   </si>
   <si>
-    <t xml:space="preserve">Damar Hamlin</t>
+    <t xml:space="preserve">DeShon Elliott</t>
   </si>
   <si>
     <t xml:space="preserve">Ernest Jones</t>
@@ -590,7 +593,7 @@
     <t xml:space="preserve">Micah Parsons</t>
   </si>
   <si>
-    <t xml:space="preserve">DeShon Elliott</t>
+    <t xml:space="preserve">Byron Murphy II</t>
   </si>
   <si>
     <t xml:space="preserve">Azeez Al-Shaair</t>
@@ -608,7 +611,7 @@
     <t xml:space="preserve">Dante Fowler Jr.</t>
   </si>
   <si>
-    <t xml:space="preserve">Byron Murphy II</t>
+    <t xml:space="preserve">Jalen Carter</t>
   </si>
   <si>
     <t xml:space="preserve">Ivan Pace Jr.</t>
@@ -626,7 +629,7 @@
     <t xml:space="preserve">B.J. Hill</t>
   </si>
   <si>
-    <t xml:space="preserve">Jalen Carter</t>
+    <t xml:space="preserve">Za’Darius Smith</t>
   </si>
   <si>
     <t xml:space="preserve">Cody Barton</t>
@@ -644,7 +647,7 @@
     <t xml:space="preserve">Nik Bonitto</t>
   </si>
   <si>
-    <t xml:space="preserve">Za’Darius Smith</t>
+    <t xml:space="preserve">Jamien Sherwood</t>
   </si>
   <si>
     <t xml:space="preserve">Alim McNeil</t>
@@ -659,7 +662,7 @@
     <t xml:space="preserve">Micah McFadden</t>
   </si>
   <si>
-    <t xml:space="preserve">Jamien Sherwood</t>
+    <t xml:space="preserve">Daiyan Henley</t>
   </si>
   <si>
     <t xml:space="preserve">Akeem Davis-Gaither</t>
@@ -671,7 +674,7 @@
     <t xml:space="preserve">Dorian Williams</t>
   </si>
   <si>
-    <t xml:space="preserve">Daiyan Henley</t>
+    <t xml:space="preserve">Patrick Queen</t>
   </si>
   <si>
     <t xml:space="preserve">Drue Tranquill</t>
@@ -683,7 +686,7 @@
     <t xml:space="preserve">Lavonte David</t>
   </si>
   <si>
-    <t xml:space="preserve">Patrick Queen</t>
+    <t xml:space="preserve">Dallas Turner</t>
   </si>
   <si>
     <t xml:space="preserve">Tryrice Knight</t>
@@ -695,15 +698,12 @@
     <t xml:space="preserve">Alex Anzalone</t>
   </si>
   <si>
-    <t xml:space="preserve">Dallas Turner</t>
+    <t xml:space="preserve">DeMavion Overshown</t>
   </si>
   <si>
     <t xml:space="preserve">Bobby Okereke</t>
   </si>
   <si>
-    <t xml:space="preserve">DeMavion Overshown</t>
-  </si>
-  <si>
     <t xml:space="preserve">Jonathoan Greenard</t>
   </si>
   <si>
@@ -1463,369 +1463,369 @@
     <t xml:space="preserve">2026 1 John O</t>
   </si>
   <si>
+    <t xml:space="preserve">2025 3 3.09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 1 Adam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 1 Ben</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 5 5.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 1 Jared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 1 Matt H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 1 Alan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 1 Josh</t>
+  </si>
+  <si>
     <t xml:space="preserve">2025 3 3.12</t>
   </si>
   <si>
-    <t xml:space="preserve">2026 1 Adam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 1 Ben</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 5 5.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 1 Jared</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 1 Matt H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 1 Alan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 1 Josh</t>
+    <t xml:space="preserve">2026 2 Adam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2 2.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 Ben</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 Jared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2 2.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 Matt H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 Alan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 John O</t>
   </si>
   <si>
     <t xml:space="preserve">2025 4 4.12</t>
   </si>
   <si>
-    <t xml:space="preserve">2026 2 Adam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2 2.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 2 Ben</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 2 Jared</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2 2.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 2 Matt H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 2 Alan</t>
+    <t xml:space="preserve">2026 3 Adam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 3 3.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 3 Ben</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 3 Jared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 3 3.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 3 Matt H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 3 Alan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 Josh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 4 4.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 Adam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 4 4.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 Ben</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 Jared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 4 4.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 Matt H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 Alan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 CJ Perry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 4 4.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 5 Adam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 5 5.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 5 Ben</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 5 Jared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 5 5.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 5 Matt H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 3 3.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 5 Alan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 John O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 5 John O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 5 5.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 4 4.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 4 4.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 5 5.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Josh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vanja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rhode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joe Luke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brandon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CJ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2 2.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 1 Vanja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 1 Rhode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 1 Joe Luke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 1 Brandon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 1 CJ Perry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2 2.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 3 3.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 Vanja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 Rhode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 Joe Luke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 Brandon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 3 John O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2 2.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 3 Josh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 3 Vanja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 3.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 3 Rhode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 3.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 3 Joe Luke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 3.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 3 Brandon</t>
   </si>
   <si>
     <t xml:space="preserve">2025 2 2.07</t>
   </si>
   <si>
-    <t xml:space="preserve">2026 2 John O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 4 4.05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 Adam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3 3.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 Ben</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 Jared</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3 3.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 Matt H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 Alan</t>
+    <t xml:space="preserve">2026 3 CJ Perry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2 2.09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 Josh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 Vanja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 4.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 Rhode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 4.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 Joe Luke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 4.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 Brandon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 4 CJ Perry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2 2.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 5 Josh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 5 Vanja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 5.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 5 Rhode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 5.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 5 Joe Luke</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 5.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 5 Brandon</t>
   </si>
   <si>
     <t xml:space="preserve">2025 3 3.05</t>
   </si>
   <si>
-    <t xml:space="preserve">2026 2 Josh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 4 4.06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 4 Adam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 4 4.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 4 Ben</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 4 Jared</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 4 4.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 4 Matt H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3 3.09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 4 Alan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 John O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 5 Adam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 5 5.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 5 Ben</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 5 Jared</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 5 5.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 5 Matt H</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3 3.06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 5 Alan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 4 John O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 5 5.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 5 John O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 4 4.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 4 4.07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 5 5.07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Josh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vanja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rhode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joe Luke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brandon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CJ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2 2.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 1 Vanja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 1 Rhode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 1 Joe Luke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 1 Brandon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 1 CJ Perry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2 2.05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3 3.07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 2 Vanja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 2 Rhode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 2 Joe Luke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 2 Brandon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 2 CJ Perry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2 2.06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 Josh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 Vanja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 Rhode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 Joe Luke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 Brandon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 3 CJ Perry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2 2.09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 4 Josh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 4 Vanja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 4.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 4 Rhode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 4.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 4 Joe Luke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 4.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 4 Brandon</t>
+    <t xml:space="preserve">2026 5 CJ Perry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 3 3.11</t>
   </si>
   <si>
     <t xml:space="preserve">2025 4.1</t>
   </si>
   <si>
-    <t xml:space="preserve">2026 4 CJ Perry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2 2.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 5 Josh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 5 Vanja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 5.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 5 Rhode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 5.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 5 Joe Luke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 5.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 5 Brandon</t>
+    <t xml:space="preserve">2025 5 5.06</t>
   </si>
   <si>
     <t xml:space="preserve">2025 5.1</t>
   </si>
   <si>
-    <t xml:space="preserve">2026 5 CJ Perry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3 3.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 5 5.06</t>
-  </si>
-  <si>
     <t xml:space="preserve">2025 5 5.05</t>
   </si>
   <si>
@@ -1884,6 +1884,15 @@
   </si>
   <si>
     <t xml:space="preserve">2025 3.09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 3 JohnO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 2 CJ</t>
   </si>
   <si>
     <t xml:space="preserve">2026 pick trades</t>
@@ -3012,387 +3021,386 @@
       <c r="V22" s="8" t="s">
         <v>102</v>
       </c>
+      <c r="W22" s="5" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="10"/>
       <c r="C23" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>102</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J23" s="7"/>
       <c r="K23" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="N23" s="10" t="s">
         <v>140</v>
       </c>
       <c r="O23" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="R23" s="8"/>
       <c r="S23" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="V23" s="8"/>
       <c r="W23" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="10"/>
       <c r="C24" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F24" s="8"/>
       <c r="G24" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J24" s="8" t="s">
         <v>102</v>
       </c>
       <c r="K24" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N24" s="10"/>
       <c r="O24" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="R24" s="8"/>
       <c r="S24" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="V24" s="8"/>
-      <c r="W24" s="5" t="s">
-        <v>157</v>
+      <c r="W24" s="0" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="10"/>
       <c r="C25" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F25" s="8"/>
       <c r="G25" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J25" s="8"/>
       <c r="K25" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N25" s="10"/>
       <c r="O25" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="R25" s="9" t="s">
         <v>121</v>
       </c>
       <c r="S25" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="V25" s="8"/>
-      <c r="W25" s="0" t="s">
         <v>163</v>
+      </c>
+      <c r="V25" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="W25" s="5" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="10"/>
       <c r="C26" s="5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F26" s="8"/>
       <c r="G26" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="J26" s="8"/>
       <c r="K26" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="N26" s="10"/>
       <c r="O26" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="R26" s="9"/>
       <c r="S26" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="V26" s="9" t="s">
-        <v>121</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="V26" s="9"/>
       <c r="W26" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>121</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J27" s="9" t="s">
         <v>121</v>
       </c>
       <c r="K27" s="0" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N27" s="10"/>
       <c r="O27" s="0" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="R27" s="9"/>
       <c r="S27" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="V27" s="9"/>
       <c r="W27" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="11"/>
       <c r="C28" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="12" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J28" s="9"/>
       <c r="K28" s="0" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="N28" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="O28" s="0" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="R28" s="9"/>
       <c r="S28" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="V28" s="9"/>
-      <c r="W28" s="5" t="s">
-        <v>182</v>
+      <c r="W28" s="0" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="11"/>
       <c r="C29" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J29" s="10" t="s">
         <v>140</v>
       </c>
       <c r="K29" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="N29" s="11"/>
       <c r="O29" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="R29" s="10" t="s">
         <v>140</v>
       </c>
       <c r="S29" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="V29" s="9"/>
-      <c r="W29" s="0" t="s">
         <v>188</v>
+      </c>
+      <c r="V29" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="W29" s="5" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="11"/>
       <c r="C30" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F30" s="10" t="s">
         <v>140</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J30" s="10"/>
       <c r="K30" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="N30" s="11"/>
       <c r="O30" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="R30" s="10"/>
       <c r="S30" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="V30" s="10" t="s">
-        <v>140</v>
-      </c>
+        <v>194</v>
+      </c>
+      <c r="V30" s="10"/>
       <c r="W30" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AB30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="11"/>
       <c r="C31" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F31" s="10"/>
       <c r="G31" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J31" s="10"/>
       <c r="K31" s="0" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="N31" s="11"/>
       <c r="O31" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="R31" s="10"/>
       <c r="S31" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="V31" s="10"/>
-      <c r="W31" s="5" t="s">
-        <v>200</v>
+      <c r="W31" s="0" t="s">
+        <v>201</v>
       </c>
       <c r="AB31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="11"/>
       <c r="C32" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F32" s="10"/>
       <c r="G32" s="0" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="J32" s="10"/>
       <c r="K32" s="12" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="N32" s="11"/>
       <c r="O32" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="R32" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S32" s="0" t="s">
-        <v>205</v>
-      </c>
-      <c r="V32" s="10"/>
-      <c r="W32" s="0" t="s">
         <v>206</v>
+      </c>
+      <c r="V32" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="W32" s="5" t="s">
+        <v>207</v>
       </c>
       <c r="AB32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F33" s="10"/>
       <c r="G33" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K33" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N33" s="11"/>
       <c r="O33" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="R33" s="11"/>
       <c r="S33" s="0" t="s">
-        <v>210</v>
-      </c>
-      <c r="V33" s="11" t="s">
-        <v>170</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="V33" s="11"/>
       <c r="W33" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F34" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G34" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J34" s="11"/>
       <c r="K34" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="R34" s="11"/>
       <c r="S34" s="0" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="V34" s="11"/>
       <c r="W34" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F35" s="11"/>
       <c r="G35" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J35" s="11"/>
       <c r="K35" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="R35" s="11"/>
       <c r="S35" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="V35" s="11"/>
-      <c r="W35" s="5" t="s">
-        <v>219</v>
+      <c r="W35" s="0" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F36" s="11"/>
       <c r="G36" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J36" s="11"/>
       <c r="K36" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="R36" s="11"/>
       <c r="S36" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="V36" s="11"/>
       <c r="W36" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F37" s="11"/>
       <c r="G37" s="0" t="s">
-        <v>224</v>
-      </c>
-      <c r="V37" s="11"/>
-      <c r="W37" s="0" t="s">
         <v>225</v>
       </c>
     </row>
@@ -4250,7 +4258,7 @@
         <v>403</v>
       </c>
       <c r="N74" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="O74" s="0" t="s">
         <v>404</v>
@@ -4304,7 +4312,7 @@
         <v>414</v>
       </c>
       <c r="J76" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K76" s="5" t="s">
         <v>415</v>
@@ -4325,13 +4333,13 @@
     </row>
     <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="16" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C77" s="0" t="s">
         <v>419</v>
       </c>
       <c r="F77" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G77" s="5" t="s">
         <v>420</v>
@@ -4371,13 +4379,13 @@
         <v>428</v>
       </c>
       <c r="R78" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="S78" s="0" t="s">
         <v>429</v>
       </c>
       <c r="V78" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="W78" s="0" t="s">
         <v>430</v>
@@ -4492,22 +4500,22 @@
     <mergeCell ref="N20:N22"/>
     <mergeCell ref="R21:R24"/>
     <mergeCell ref="B22:B26"/>
-    <mergeCell ref="V22:V25"/>
+    <mergeCell ref="V22:V24"/>
     <mergeCell ref="F23:F26"/>
     <mergeCell ref="N23:N27"/>
     <mergeCell ref="J24:J26"/>
     <mergeCell ref="R25:R28"/>
-    <mergeCell ref="V26:V29"/>
+    <mergeCell ref="V25:V28"/>
     <mergeCell ref="F27:F29"/>
     <mergeCell ref="J27:J28"/>
     <mergeCell ref="N28:N33"/>
     <mergeCell ref="J29:J32"/>
     <mergeCell ref="R29:R31"/>
+    <mergeCell ref="V29:V31"/>
     <mergeCell ref="F30:F33"/>
-    <mergeCell ref="V30:V32"/>
     <mergeCell ref="R32:R36"/>
+    <mergeCell ref="V32:V36"/>
     <mergeCell ref="J33:J36"/>
-    <mergeCell ref="V33:V37"/>
     <mergeCell ref="F34:F38"/>
     <mergeCell ref="B45:C45"/>
     <mergeCell ref="F45:G45"/>
@@ -4853,140 +4861,134 @@
       <c r="BG3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="B4" s="0" t="s">
         <v>500</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="D4" s="0" t="s">
         <v>501</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="E4" s="0" t="s">
         <v>502</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="G4" s="0" t="s">
         <v>503</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="H4" s="0" t="s">
         <v>504</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="K4" s="0" t="s">
         <v>505</v>
       </c>
-      <c r="K4" s="0" t="s">
+      <c r="M4" s="0" t="s">
         <v>506</v>
       </c>
-      <c r="M4" s="0" t="s">
+      <c r="N4" s="0" t="s">
         <v>507</v>
       </c>
-      <c r="N4" s="0" t="s">
+      <c r="P4" s="5" t="s">
         <v>508</v>
       </c>
-      <c r="P4" s="5" t="s">
+      <c r="Q4" s="0" t="s">
         <v>509</v>
       </c>
-      <c r="Q4" s="0" t="s">
+      <c r="BG4" s="0"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="0" t="s">
         <v>510</v>
       </c>
-      <c r="BG4" s="0"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="D5" s="0" t="s">
         <v>511</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="E5" s="0" t="s">
         <v>512</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="G5" s="0" t="s">
         <v>513</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="H5" s="0" t="s">
         <v>514</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="K5" s="0" t="s">
         <v>515</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="M5" s="0" t="s">
         <v>516</v>
       </c>
-      <c r="K5" s="0" t="s">
+      <c r="N5" s="0" t="s">
         <v>517</v>
       </c>
-      <c r="M5" s="0" t="s">
+      <c r="Q5" s="0" t="s">
         <v>518</v>
-      </c>
-      <c r="N5" s="0" t="s">
-        <v>519</v>
-      </c>
-      <c r="P5" s="0" t="s">
-        <v>520</v>
-      </c>
-      <c r="Q5" s="0" t="s">
-        <v>521</v>
       </c>
       <c r="BG5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
+        <v>519</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>520</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>521</v>
+      </c>
+      <c r="G6" s="0" t="s">
         <v>522</v>
       </c>
-      <c r="D6" s="0" t="s">
-        <v>483</v>
-      </c>
-      <c r="E6" s="0" t="s">
+      <c r="H6" s="0" t="s">
         <v>523</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="K6" s="0" t="s">
         <v>524</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="M6" s="0" t="s">
         <v>525</v>
       </c>
-      <c r="K6" s="0" t="s">
+      <c r="N6" s="0" t="s">
         <v>526</v>
       </c>
-      <c r="M6" s="0" t="s">
+      <c r="P6" s="0" t="s">
         <v>527</v>
       </c>
-      <c r="N6" s="0" t="s">
+      <c r="Q6" s="0" t="s">
         <v>528</v>
-      </c>
-      <c r="P6" s="0" t="s">
-        <v>529</v>
-      </c>
-      <c r="Q6" s="0" t="s">
-        <v>530</v>
       </c>
       <c r="BG6" s="0"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>532</v>
+        <v>483</v>
       </c>
       <c r="P7" s="0" t="s">
-        <v>513</v>
+        <v>520</v>
       </c>
       <c r="BG7" s="0"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>533</v>
+        <v>530</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>531</v>
       </c>
       <c r="P8" s="0" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="BG8" s="0"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P9" s="0" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="BG9" s="0"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P10" s="0" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="BG10" s="0"/>
     </row>
@@ -5022,230 +5024,235 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="B21" s="1"/>
       <c r="D21" s="1" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="19"/>
       <c r="G21" s="1" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="H21" s="1"/>
       <c r="J21" s="1" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="K21" s="1"/>
       <c r="L21" s="19"/>
       <c r="M21" s="1" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="N21" s="1"/>
       <c r="P21" s="1" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="Q21" s="1"/>
       <c r="BG21" s="0"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
+        <v>541</v>
+      </c>
+      <c r="D22" s="0" t="s">
+        <v>542</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>543</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="G22" s="5" t="s">
         <v>544</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="H22" s="5" t="s">
         <v>545</v>
       </c>
-      <c r="G22" s="5" t="s">
+      <c r="J22" s="5" t="s">
         <v>546</v>
       </c>
-      <c r="H22" s="5" t="s">
+      <c r="K22" s="5" t="s">
         <v>547</v>
       </c>
-      <c r="J22" s="5" t="s">
+      <c r="M22" s="5" t="s">
         <v>548</v>
       </c>
-      <c r="K22" s="5" t="s">
+      <c r="N22" s="5" t="s">
         <v>549</v>
       </c>
-      <c r="M22" s="5" t="s">
+      <c r="P22" s="5" t="s">
         <v>550</v>
       </c>
-      <c r="N22" s="5" t="s">
+      <c r="Q22" s="5" t="s">
         <v>551</v>
-      </c>
-      <c r="P22" s="5" t="s">
-        <v>552</v>
-      </c>
-      <c r="Q22" s="5" t="s">
-        <v>553</v>
       </c>
       <c r="BG22" s="0"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
+        <v>552</v>
+      </c>
+      <c r="D23" s="0" t="s">
+        <v>553</v>
+      </c>
+      <c r="E23" s="0" t="s">
         <v>554</v>
       </c>
-      <c r="D23" s="0" t="s">
+      <c r="G23" s="0" t="s">
         <v>555</v>
       </c>
-      <c r="E23" s="0" t="s">
+      <c r="H23" s="0" t="s">
         <v>556</v>
       </c>
-      <c r="G23" s="0" t="s">
+      <c r="J23" s="0" t="s">
         <v>557</v>
       </c>
-      <c r="H23" s="0" t="s">
+      <c r="K23" s="0" t="s">
         <v>558</v>
       </c>
-      <c r="J23" s="0" t="s">
+      <c r="M23" s="0" t="s">
         <v>559</v>
       </c>
-      <c r="K23" s="0" t="s">
+      <c r="N23" s="0" t="s">
         <v>560</v>
       </c>
-      <c r="M23" s="0" t="s">
+      <c r="P23" s="0" t="s">
         <v>561</v>
       </c>
-      <c r="N23" s="0" t="s">
+      <c r="Q23" s="0" t="s">
         <v>562</v>
-      </c>
-      <c r="P23" s="0" t="s">
-        <v>563</v>
-      </c>
-      <c r="Q23" s="0" t="s">
-        <v>564</v>
       </c>
       <c r="BG23" s="0"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
+        <v>563</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>564</v>
+      </c>
+      <c r="E24" s="0" t="s">
         <v>565</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="G24" s="0" t="s">
         <v>566</v>
       </c>
-      <c r="E24" s="0" t="s">
+      <c r="H24" s="0" t="s">
         <v>567</v>
       </c>
-      <c r="G24" s="0" t="s">
+      <c r="J24" s="0" t="s">
         <v>568</v>
       </c>
-      <c r="H24" s="0" t="s">
+      <c r="K24" s="0" t="s">
         <v>569</v>
       </c>
-      <c r="J24" s="0" t="s">
+      <c r="M24" s="0" t="s">
         <v>570</v>
       </c>
-      <c r="K24" s="0" t="s">
+      <c r="N24" s="0" t="s">
         <v>571</v>
       </c>
-      <c r="M24" s="0" t="s">
+      <c r="P24" s="0" t="s">
         <v>572</v>
       </c>
-      <c r="N24" s="0" t="s">
+      <c r="Q24" s="0" t="s">
         <v>573</v>
-      </c>
-      <c r="P24" s="0" t="s">
-        <v>574</v>
-      </c>
-      <c r="Q24" s="0" t="s">
-        <v>575</v>
       </c>
       <c r="BG24" s="0"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
+        <v>574</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>575</v>
+      </c>
+      <c r="E25" s="0" t="s">
         <v>576</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="G25" s="0" t="s">
         <v>577</v>
       </c>
-      <c r="E25" s="0" t="s">
+      <c r="H25" s="0" t="s">
         <v>578</v>
       </c>
-      <c r="G25" s="0" t="s">
+      <c r="J25" s="0" t="s">
         <v>579</v>
       </c>
-      <c r="H25" s="0" t="s">
+      <c r="K25" s="0" t="s">
         <v>580</v>
       </c>
-      <c r="J25" s="0" t="s">
+      <c r="M25" s="0" t="s">
         <v>581</v>
       </c>
-      <c r="K25" s="0" t="s">
+      <c r="N25" s="0" t="s">
         <v>582</v>
       </c>
-      <c r="M25" s="0" t="s">
+      <c r="P25" s="0" t="s">
         <v>583</v>
       </c>
-      <c r="N25" s="0" t="s">
+      <c r="Q25" s="0" t="s">
         <v>584</v>
-      </c>
-      <c r="P25" s="0" t="s">
-        <v>585</v>
-      </c>
-      <c r="Q25" s="0" t="s">
-        <v>586</v>
       </c>
       <c r="BG25" s="0"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
+        <v>585</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>586</v>
+      </c>
+      <c r="E26" s="0" t="s">
         <v>587</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="G26" s="0" t="s">
         <v>588</v>
       </c>
-      <c r="E26" s="0" t="s">
+      <c r="H26" s="0" t="s">
         <v>589</v>
       </c>
-      <c r="G26" s="0" t="s">
+      <c r="J26" s="0" t="s">
         <v>590</v>
       </c>
-      <c r="H26" s="0" t="s">
+      <c r="K26" s="0" t="s">
         <v>591</v>
       </c>
-      <c r="J26" s="0" t="s">
+      <c r="M26" s="0" t="s">
         <v>592</v>
       </c>
-      <c r="K26" s="0" t="s">
+      <c r="N26" s="0" t="s">
         <v>593</v>
       </c>
-      <c r="M26" s="0" t="s">
+      <c r="P26" s="0" t="s">
         <v>594</v>
       </c>
-      <c r="N26" s="0" t="s">
+      <c r="Q26" s="0" t="s">
         <v>595</v>
-      </c>
-      <c r="P26" s="0" t="s">
-        <v>596</v>
-      </c>
-      <c r="Q26" s="0" t="s">
-        <v>597</v>
       </c>
       <c r="BG26" s="0"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="D27" s="5"/>
       <c r="G27" s="5"/>
       <c r="J27" s="5"/>
       <c r="M27" s="5"/>
-      <c r="P27" s="5"/>
+      <c r="P27" s="0" t="s">
+        <v>597</v>
+      </c>
       <c r="BG27" s="0"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="G28" s="5"/>
       <c r="M28" s="5"/>
+      <c r="P28" s="0" t="s">
+        <v>599</v>
+      </c>
       <c r="BG28" s="0"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7159,7 +7166,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="23" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="B1" s="24" t="s">
         <v>609</v>
@@ -7179,7 +7186,7 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="25" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="B4" s="26" t="s">
         <v>324</v>
@@ -7205,7 +7212,7 @@
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="B9" s="24" t="s">
         <v>612</v>
@@ -7220,7 +7227,7 @@
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27"/>
       <c r="B11" s="28" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7255,10 +7262,10 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7297,7 +7304,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="B25" s="24" t="s">
         <v>618</v>
@@ -7345,13 +7352,45 @@
         <v>476</v>
       </c>
       <c r="B33" s="30" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="27"/>
       <c r="B34" s="28" t="s">
         <v>619</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="23" t="s">
+        <v>613</v>
+      </c>
+      <c r="B36" s="29" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="25"/>
+      <c r="B37" s="30" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="25"/>
+      <c r="B38" s="30" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="25"/>
+      <c r="B39" s="30"/>
+    </row>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="27" t="s">
+        <v>540</v>
+      </c>
+      <c r="B40" s="28" t="s">
+        <v>622</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7521,7 +7560,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="32" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="B1" s="32"/>
     </row>

</xml_diff>

<commit_message>
picks and uploaded to yahoo
</commit_message>
<xml_diff>
--- a/OffSeason.xlsx
+++ b/OffSeason.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Rosters" sheetId="1" state="visible" r:id="rId2"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="628">
   <si>
     <t xml:space="preserve">No Chubb – John Olson</t>
   </si>
@@ -557,129 +557,155 @@
     <t xml:space="preserve">Will Anderson</t>
   </si>
   <si>
+    <t xml:space="preserve">2025 3 3.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fred Warner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carl Granderson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Micah McFadden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dallas Turner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noah Brown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zack Baun</t>
+  </si>
+  <si>
     <t xml:space="preserve">2025 3 3.09</t>
   </si>
   <si>
-    <t xml:space="preserve">Fred Warner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carl Granderson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Micah McFadden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dallas Turner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noah Brown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zack Baun</t>
+    <t xml:space="preserve">Kaden Ellis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Danielle Hunter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lavonte David</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A’Shawn Robinson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roquan Smith</t>
   </si>
   <si>
     <t xml:space="preserve">2025 3 3.12</t>
   </si>
   <si>
-    <t xml:space="preserve">Kaden Ellis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Danielle Hunter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lavonte David</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A’Shawn Robinson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roquan Smith</t>
+    <t xml:space="preserve">2025 1 1.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calijah Kancey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alex Anzalone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.09</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">End 26</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">th</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Henry To’oTo’o</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ernest Jones</t>
   </si>
   <si>
     <t xml:space="preserve">2025 4 4.12</t>
   </si>
   <si>
-    <t xml:space="preserve">2025 1 1.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calijah Kancey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alex Anzalone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Henry To’oTo’o</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ernest Jones</t>
+    <t xml:space="preserve">2025 2 2.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quay Walker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quintin Lake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ivan Pace Jr.</t>
   </si>
   <si>
     <t xml:space="preserve">2025 4 4.05</t>
   </si>
   <si>
-    <t xml:space="preserve">2025 2 2.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quay Walker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quintin Lake</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ivan Pace Jr.</t>
+    <t xml:space="preserve">2025 3 3.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foyesade Oluokun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 2 2.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 3 3.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Junior Colson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 1 1.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 5 5.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 4 4.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logan Wilson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 3 3.08</t>
   </si>
   <si>
     <t xml:space="preserve">2025 4 4.06</t>
   </si>
   <si>
-    <t xml:space="preserve">2025 3 3.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Foyesade Oluokun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 2 2.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3 3.06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Junior Colson</t>
+    <t xml:space="preserve">Taysom Hill (QB/TE</t>
   </si>
   <si>
     <t xml:space="preserve">2025 1 1.11</t>
   </si>
   <si>
-    <t xml:space="preserve">2025 5 5.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 4 4.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logan Wilson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 3 3.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Taysom Hill (QB/TE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025 1 1.07</t>
-  </si>
-  <si>
     <t xml:space="preserve">2025 5 5.12</t>
   </si>
   <si>
@@ -704,6 +730,9 @@
     <t xml:space="preserve">Raheem Mostert</t>
   </si>
   <si>
+    <t xml:space="preserve">issue keepers</t>
+  </si>
+  <si>
     <t xml:space="preserve">Trey Sermon</t>
   </si>
   <si>
@@ -1757,9 +1786,6 @@
     <t xml:space="preserve">2026 4 CJ Perry</t>
   </si>
   <si>
-    <t xml:space="preserve">2025 3 3.07</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026 2 Vanja</t>
   </si>
   <si>
@@ -1827,6 +1853,12 @@
   </si>
   <si>
     <t xml:space="preserve">2026 5 CJ Perry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 6.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025 7.3</t>
   </si>
   <si>
     <t xml:space="preserve">2025 picks</t>
@@ -1907,7 +1939,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1942,6 +1974,14 @@
       <b val="true"/>
       <i val="true"/>
       <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <vertAlign val="superscript"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -2132,7 +2172,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
@@ -2189,12 +2229,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2205,11 +2245,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2217,7 +2257,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2265,11 +2305,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3666,7 +3706,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="n">
         <v>26</v>
       </c>
@@ -3706,8 +3746,11 @@
       <c r="W27" s="5" t="s">
         <v>195</v>
       </c>
+      <c r="X27" s="0" t="s">
+        <v>196</v>
+      </c>
       <c r="AB27" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3716,19 +3759,19 @@
       </c>
       <c r="B28" s="11"/>
       <c r="C28" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E28" s="0" t="n">
         <v>27</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I28" s="0" t="n">
         <v>27</v>
       </c>
       <c r="K28" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M28" s="0" t="n">
         <v>27</v>
@@ -3737,22 +3780,22 @@
         <v>148</v>
       </c>
       <c r="O28" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="Q28" s="0" t="n">
         <v>27</v>
       </c>
       <c r="S28" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="U28" s="0" t="n">
         <v>27</v>
       </c>
       <c r="W28" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AB28" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3761,41 +3804,41 @@
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E29" s="0" t="n">
         <v>28</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I29" s="0" t="n">
         <v>28</v>
       </c>
       <c r="K29" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="M29" s="0" t="n">
         <v>28</v>
       </c>
       <c r="N29" s="11"/>
       <c r="O29" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="Q29" s="0" t="n">
         <v>28</v>
       </c>
       <c r="S29" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="U29" s="0" t="n">
         <v>28</v>
       </c>
       <c r="W29" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="AB29" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3803,41 +3846,41 @@
         <v>29</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E30" s="0" t="n">
         <v>29</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="I30" s="0" t="n">
         <v>29</v>
       </c>
       <c r="K30" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="M30" s="0" t="n">
         <v>29</v>
       </c>
       <c r="N30" s="11"/>
       <c r="O30" s="5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Q30" s="0" t="n">
         <v>29</v>
       </c>
       <c r="S30" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="U30" s="0" t="n">
         <v>29</v>
       </c>
       <c r="W30" s="0" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="AB30" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3845,139 +3888,142 @@
         <v>30</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E31" s="0" t="n">
         <v>30</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="I31" s="0" t="n">
         <v>30</v>
       </c>
       <c r="K31" s="0" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="M31" s="0" t="n">
         <v>30</v>
       </c>
       <c r="N31" s="11"/>
       <c r="O31" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="Q31" s="0" t="n">
         <v>30</v>
       </c>
       <c r="S31" s="0" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="U31" s="0" t="n">
         <v>30</v>
       </c>
       <c r="W31" s="0" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AB31" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB32" s="5" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB33" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="W34" s="13" t="s">
+        <v>228</v>
+      </c>
       <c r="AB34" s="5" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB35" s="5" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB36" s="5" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB37" s="5" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="S38" s="5"/>
       <c r="AB38" s="5" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB39" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB40" s="0" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB41" s="12" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB42" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="13"/>
-      <c r="H43" s="13"/>
+      <c r="B43" s="14"/>
+      <c r="H43" s="14"/>
       <c r="AB43" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="13"/>
+      <c r="B44" s="14"/>
       <c r="AB44" s="5" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="1" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C45" s="1"/>
       <c r="F45" s="1" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="G45" s="1"/>
       <c r="J45" s="1" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="K45" s="1"/>
       <c r="N45" s="1" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="O45" s="1"/>
       <c r="R45" s="1" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="S45" s="1"/>
       <c r="V45" s="1" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="W45" s="1"/>
       <c r="AB45" s="5" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3988,7 +4034,7 @@
         <v>7</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="E46" s="0" t="n">
         <v>1</v>
@@ -3997,7 +4043,7 @@
         <v>7</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I46" s="0" t="n">
         <v>1</v>
@@ -4006,7 +4052,7 @@
         <v>7</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="M46" s="0" t="n">
         <v>1</v>
@@ -4015,7 +4061,7 @@
         <v>7</v>
       </c>
       <c r="O46" s="5" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="Q46" s="0" t="n">
         <v>1</v>
@@ -4024,7 +4070,7 @@
         <v>7</v>
       </c>
       <c r="S46" s="5" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="U46" s="0" t="n">
         <v>1</v>
@@ -4033,10 +4079,10 @@
         <v>7</v>
       </c>
       <c r="W46" s="5" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="AB46" s="5" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4045,45 +4091,45 @@
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="5" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E47" s="0" t="n">
         <v>2</v>
       </c>
       <c r="F47" s="4"/>
       <c r="G47" s="5" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="I47" s="0" t="n">
         <v>2</v>
       </c>
       <c r="J47" s="4"/>
       <c r="K47" s="5" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="M47" s="0" t="n">
         <v>2</v>
       </c>
       <c r="N47" s="4"/>
       <c r="O47" s="5" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="Q47" s="0" t="n">
         <v>2</v>
       </c>
       <c r="R47" s="4"/>
       <c r="S47" s="5" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="U47" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="V47" s="14"/>
+      <c r="V47" s="13"/>
       <c r="W47" s="5" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="AB47" s="5" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4092,21 +4138,21 @@
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="5" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E48" s="0" t="n">
         <v>3</v>
       </c>
       <c r="F48" s="4"/>
       <c r="G48" s="5" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="I48" s="0" t="n">
         <v>3</v>
       </c>
       <c r="J48" s="4"/>
       <c r="K48" s="5" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="M48" s="0" t="n">
         <v>3</v>
@@ -4115,14 +4161,14 @@
         <v>22</v>
       </c>
       <c r="O48" s="5" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="Q48" s="0" t="n">
         <v>3</v>
       </c>
       <c r="R48" s="4"/>
       <c r="S48" s="5" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="U48" s="0" t="n">
         <v>3</v>
@@ -4131,10 +4177,10 @@
         <v>22</v>
       </c>
       <c r="W48" s="5" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="AB48" s="5" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4145,7 +4191,7 @@
         <v>22</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="E49" s="0" t="n">
         <v>4</v>
@@ -4154,7 +4200,7 @@
         <v>22</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="I49" s="0" t="n">
         <v>4</v>
@@ -4163,31 +4209,31 @@
         <v>22</v>
       </c>
       <c r="K49" s="5" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="M49" s="0" t="n">
         <v>4</v>
       </c>
       <c r="N49" s="6"/>
       <c r="O49" s="5" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="Q49" s="0" t="n">
         <v>4</v>
       </c>
       <c r="R49" s="4"/>
       <c r="S49" s="0" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="U49" s="0" t="n">
         <v>4</v>
       </c>
       <c r="V49" s="6"/>
       <c r="W49" s="5" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="AB49" s="5" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4196,28 +4242,28 @@
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="5" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="E50" s="0" t="n">
         <v>5</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="5" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="I50" s="0" t="n">
         <v>5</v>
       </c>
       <c r="J50" s="6"/>
       <c r="K50" s="5" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="M50" s="0" t="n">
         <v>5</v>
       </c>
       <c r="N50" s="6"/>
       <c r="O50" s="5" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="Q50" s="0" t="n">
         <v>5</v>
@@ -4226,17 +4272,17 @@
         <v>22</v>
       </c>
       <c r="S50" s="5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="U50" s="0" t="n">
         <v>5</v>
       </c>
       <c r="V50" s="6"/>
       <c r="W50" s="5" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="AB50" s="5" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4245,35 +4291,35 @@
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="0" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E51" s="0" t="n">
         <v>6</v>
       </c>
       <c r="F51" s="6"/>
       <c r="G51" s="5" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="I51" s="0" t="n">
         <v>6</v>
       </c>
       <c r="J51" s="6"/>
       <c r="K51" s="5" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="M51" s="0" t="n">
         <v>6</v>
       </c>
       <c r="N51" s="6"/>
       <c r="O51" s="5" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="Q51" s="0" t="n">
         <v>6</v>
       </c>
       <c r="R51" s="6"/>
       <c r="S51" s="5" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="U51" s="0" t="n">
         <v>6</v>
@@ -4282,10 +4328,10 @@
         <v>45</v>
       </c>
       <c r="W51" s="5" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="AB51" s="5" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4294,45 +4340,45 @@
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="5" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E52" s="0" t="n">
         <v>7</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="5" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="I52" s="0" t="n">
         <v>7</v>
       </c>
       <c r="J52" s="6"/>
       <c r="K52" s="5" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="M52" s="0" t="n">
         <v>7</v>
       </c>
       <c r="N52" s="6"/>
       <c r="O52" s="5" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="Q52" s="0" t="n">
         <v>7</v>
       </c>
       <c r="R52" s="6"/>
       <c r="S52" s="5" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="U52" s="0" t="n">
         <v>7</v>
       </c>
       <c r="V52" s="7"/>
       <c r="W52" s="5" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="AB52" s="0" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4341,14 +4387,14 @@
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="5" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E53" s="0" t="n">
         <v>8</v>
       </c>
       <c r="F53" s="6"/>
       <c r="G53" s="0" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="I53" s="0" t="n">
         <v>8</v>
@@ -4357,7 +4403,7 @@
         <v>45</v>
       </c>
       <c r="K53" s="5" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="M53" s="0" t="n">
         <v>8</v>
@@ -4366,24 +4412,24 @@
         <v>45</v>
       </c>
       <c r="O53" s="5" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="Q53" s="0" t="n">
         <v>8</v>
       </c>
       <c r="R53" s="6"/>
       <c r="S53" s="5" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="U53" s="0" t="n">
         <v>8</v>
       </c>
       <c r="V53" s="7"/>
       <c r="W53" s="5" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="AB53" s="0" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4394,28 +4440,28 @@
         <v>45</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="E54" s="0" t="n">
         <v>9</v>
       </c>
       <c r="F54" s="6"/>
       <c r="G54" s="5" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="I54" s="0" t="n">
         <v>9</v>
       </c>
       <c r="J54" s="7"/>
       <c r="K54" s="5" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="M54" s="0" t="n">
         <v>9</v>
       </c>
       <c r="N54" s="7"/>
       <c r="O54" s="5" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="Q54" s="0" t="n">
         <v>9</v>
@@ -4424,17 +4470,17 @@
         <v>45</v>
       </c>
       <c r="S54" s="5" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="U54" s="0" t="n">
         <v>9</v>
       </c>
       <c r="V54" s="7"/>
       <c r="W54" s="5" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="AB54" s="0" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4443,7 +4489,7 @@
       </c>
       <c r="B55" s="7"/>
       <c r="C55" s="5" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="E55" s="0" t="n">
         <v>10</v>
@@ -4452,38 +4498,38 @@
         <v>45</v>
       </c>
       <c r="G55" s="5" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="I55" s="0" t="n">
         <v>10</v>
       </c>
       <c r="J55" s="7"/>
       <c r="K55" s="5" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="M55" s="0" t="n">
         <v>10</v>
       </c>
       <c r="N55" s="7"/>
       <c r="O55" s="5" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="Q55" s="0" t="n">
         <v>10</v>
       </c>
       <c r="R55" s="7"/>
       <c r="S55" s="5" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="U55" s="0" t="n">
         <v>10</v>
       </c>
       <c r="V55" s="7"/>
       <c r="W55" s="5" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="AB55" s="5" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4492,45 +4538,45 @@
       </c>
       <c r="B56" s="7"/>
       <c r="C56" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E56" s="0" t="n">
         <v>11</v>
       </c>
       <c r="F56" s="7"/>
       <c r="G56" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="I56" s="0" t="n">
         <v>11</v>
       </c>
       <c r="J56" s="7"/>
       <c r="K56" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="M56" s="0" t="n">
         <v>11</v>
       </c>
       <c r="N56" s="7"/>
       <c r="O56" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="Q56" s="0" t="n">
         <v>11</v>
       </c>
       <c r="R56" s="7"/>
       <c r="S56" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="U56" s="0" t="n">
         <v>11</v>
       </c>
       <c r="V56" s="7"/>
       <c r="W56" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="AB56" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4539,14 +4585,14 @@
       </c>
       <c r="B57" s="7"/>
       <c r="C57" s="5" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="E57" s="0" t="n">
         <v>12</v>
       </c>
       <c r="F57" s="7"/>
       <c r="G57" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="I57" s="0" t="n">
         <v>12</v>
@@ -4555,7 +4601,7 @@
         <v>89</v>
       </c>
       <c r="K57" s="5" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="M57" s="0" t="n">
         <v>12</v>
@@ -4564,24 +4610,24 @@
         <v>89</v>
       </c>
       <c r="O57" s="5" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="Q57" s="0" t="n">
         <v>12</v>
       </c>
       <c r="R57" s="7"/>
       <c r="S57" s="5" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="U57" s="0" t="n">
         <v>12</v>
       </c>
       <c r="V57" s="7"/>
       <c r="W57" s="5" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="AB57" s="5" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4590,14 +4636,14 @@
       </c>
       <c r="B58" s="7"/>
       <c r="C58" s="5" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="E58" s="0" t="n">
         <v>13</v>
       </c>
       <c r="F58" s="7"/>
       <c r="G58" s="5" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="I58" s="0" t="n">
         <v>13</v>
@@ -4606,31 +4652,31 @@
         <v>111</v>
       </c>
       <c r="K58" s="5" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="M58" s="0" t="n">
         <v>13</v>
       </c>
       <c r="N58" s="8"/>
       <c r="O58" s="5" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="Q58" s="0" t="n">
         <v>13</v>
       </c>
       <c r="R58" s="7"/>
       <c r="S58" s="5" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="U58" s="0" t="n">
         <v>13</v>
       </c>
       <c r="V58" s="7"/>
       <c r="W58" s="5" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="AB58" s="5" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4639,21 +4685,21 @@
       </c>
       <c r="B59" s="7"/>
       <c r="C59" s="5" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="E59" s="0" t="n">
         <v>14</v>
       </c>
       <c r="F59" s="7"/>
       <c r="G59" s="5" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="I59" s="0" t="n">
         <v>14</v>
       </c>
       <c r="J59" s="9"/>
       <c r="K59" s="5" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="M59" s="0" t="n">
         <v>14</v>
@@ -4662,14 +4708,14 @@
         <v>111</v>
       </c>
       <c r="O59" s="5" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="Q59" s="0" t="n">
         <v>14</v>
       </c>
       <c r="R59" s="7"/>
       <c r="S59" s="5" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="U59" s="0" t="n">
         <v>14</v>
@@ -4678,10 +4724,10 @@
         <v>89</v>
       </c>
       <c r="W59" s="0" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="AB59" s="5" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4690,28 +4736,28 @@
       </c>
       <c r="B60" s="7"/>
       <c r="C60" s="5" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="E60" s="0" t="n">
         <v>15</v>
       </c>
       <c r="F60" s="7"/>
       <c r="G60" s="5" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="I60" s="0" t="n">
         <v>15</v>
       </c>
       <c r="J60" s="9"/>
       <c r="K60" s="5" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="M60" s="0" t="n">
         <v>15</v>
       </c>
       <c r="N60" s="9"/>
       <c r="O60" s="5" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="Q60" s="0" t="n">
         <v>15</v>
@@ -4720,17 +4766,17 @@
         <v>89</v>
       </c>
       <c r="S60" s="5" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="U60" s="0" t="n">
         <v>15</v>
       </c>
       <c r="V60" s="8"/>
       <c r="W60" s="0" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="AB60" s="5" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4741,14 +4787,14 @@
         <v>89</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="E61" s="0" t="n">
         <v>16</v>
       </c>
       <c r="F61" s="7"/>
       <c r="G61" s="0" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="I61" s="0" t="n">
         <v>16</v>
@@ -4757,7 +4803,7 @@
         <v>126</v>
       </c>
       <c r="K61" s="5" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="M61" s="0" t="n">
         <v>16</v>
@@ -4766,24 +4812,24 @@
         <v>126</v>
       </c>
       <c r="O61" s="0" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="Q61" s="0" t="n">
         <v>16</v>
       </c>
       <c r="R61" s="8"/>
       <c r="S61" s="5" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="U61" s="0" t="n">
         <v>16</v>
       </c>
       <c r="V61" s="8"/>
       <c r="W61" s="0" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="AB61" s="5" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4792,35 +4838,35 @@
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="5" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="E62" s="0" t="n">
         <v>17</v>
       </c>
       <c r="F62" s="7"/>
       <c r="G62" s="0" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="I62" s="0" t="n">
         <v>17</v>
       </c>
       <c r="J62" s="10"/>
       <c r="K62" s="5" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="M62" s="0" t="n">
         <v>17</v>
       </c>
       <c r="N62" s="10"/>
       <c r="O62" s="0" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="Q62" s="0" t="n">
         <v>17</v>
       </c>
       <c r="R62" s="8"/>
       <c r="S62" s="5" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="U62" s="0" t="n">
         <v>17</v>
@@ -4829,10 +4875,10 @@
         <v>111</v>
       </c>
       <c r="W62" s="0" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="AB62" s="5" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4843,28 +4889,28 @@
         <v>111</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="E63" s="0" t="n">
         <v>18</v>
       </c>
       <c r="F63" s="7"/>
       <c r="G63" s="5" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="I63" s="0" t="n">
         <v>18</v>
       </c>
       <c r="J63" s="10"/>
       <c r="K63" s="5" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="M63" s="0" t="n">
         <v>18</v>
       </c>
       <c r="N63" s="10"/>
       <c r="O63" s="0" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="Q63" s="0" t="n">
         <v>18</v>
@@ -4873,7 +4919,7 @@
         <v>111</v>
       </c>
       <c r="S63" s="5" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="U63" s="0" t="n">
         <v>18</v>
@@ -4882,10 +4928,10 @@
         <v>126</v>
       </c>
       <c r="W63" s="0" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="AB63" s="5" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4894,35 +4940,35 @@
       </c>
       <c r="B64" s="9"/>
       <c r="C64" s="5" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="E64" s="0" t="n">
         <v>19</v>
       </c>
       <c r="F64" s="7"/>
       <c r="G64" s="0" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="I64" s="0" t="n">
         <v>19</v>
       </c>
       <c r="J64" s="10"/>
       <c r="K64" s="5" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="M64" s="0" t="n">
         <v>19</v>
       </c>
       <c r="N64" s="10"/>
       <c r="O64" s="0" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="Q64" s="0" t="n">
         <v>19</v>
       </c>
       <c r="R64" s="9"/>
       <c r="S64" s="5" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="U64" s="0" t="n">
         <v>19</v>
@@ -4931,10 +4977,10 @@
         <v>148</v>
       </c>
       <c r="W64" s="0" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="AB64" s="0" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4943,7 +4989,7 @@
       </c>
       <c r="B65" s="9"/>
       <c r="C65" s="0" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E65" s="0" t="n">
         <v>20</v>
@@ -4952,14 +4998,14 @@
         <v>89</v>
       </c>
       <c r="G65" s="5" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="I65" s="0" t="n">
         <v>20</v>
       </c>
       <c r="J65" s="10"/>
       <c r="K65" s="5" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="M65" s="0" t="n">
         <v>20</v>
@@ -4968,7 +5014,7 @@
         <v>148</v>
       </c>
       <c r="O65" s="0" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="Q65" s="0" t="n">
         <v>20</v>
@@ -4977,17 +5023,17 @@
         <v>126</v>
       </c>
       <c r="S65" s="0" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="U65" s="0" t="n">
         <v>20</v>
       </c>
       <c r="V65" s="11"/>
       <c r="W65" s="0" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="AB65" s="5" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4998,44 +5044,44 @@
         <v>126</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="E66" s="0" t="n">
         <v>21</v>
       </c>
       <c r="F66" s="8"/>
       <c r="G66" s="5" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="I66" s="0" t="n">
         <v>21</v>
       </c>
       <c r="J66" s="10"/>
       <c r="K66" s="5" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="M66" s="0" t="n">
         <v>21</v>
       </c>
       <c r="N66" s="11"/>
       <c r="O66" s="0" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="Q66" s="0" t="n">
         <v>21</v>
       </c>
       <c r="R66" s="10"/>
       <c r="S66" s="0" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="U66" s="0" t="n">
         <v>21</v>
       </c>
       <c r="W66" s="5" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="AB66" s="0" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5044,44 +5090,44 @@
       </c>
       <c r="B67" s="10"/>
       <c r="C67" s="0" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="E67" s="0" t="n">
         <v>22</v>
       </c>
       <c r="F67" s="8"/>
       <c r="G67" s="0" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="I67" s="0" t="n">
         <v>22</v>
       </c>
       <c r="J67" s="10"/>
       <c r="K67" s="0" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="M67" s="0" t="n">
         <v>22</v>
       </c>
       <c r="N67" s="11"/>
       <c r="O67" s="0" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="Q67" s="0" t="n">
         <v>22</v>
       </c>
       <c r="R67" s="10"/>
       <c r="S67" s="0" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="U67" s="0" t="n">
         <v>22</v>
       </c>
       <c r="W67" s="0" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="AB67" s="0" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5090,7 +5136,7 @@
       </c>
       <c r="B68" s="10"/>
       <c r="C68" s="0" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E68" s="0" t="n">
         <v>23</v>
@@ -5099,7 +5145,7 @@
         <v>111</v>
       </c>
       <c r="G68" s="5" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="I68" s="0" t="n">
         <v>23</v>
@@ -5108,14 +5154,14 @@
         <v>148</v>
       </c>
       <c r="K68" s="5" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="M68" s="0" t="n">
         <v>23</v>
       </c>
       <c r="N68" s="11"/>
       <c r="O68" s="0" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="Q68" s="0" t="n">
         <v>23</v>
@@ -5124,16 +5170,16 @@
         <v>148</v>
       </c>
       <c r="S68" s="0" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="U68" s="0" t="n">
         <v>23</v>
       </c>
       <c r="W68" s="0" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="AB68" s="5" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5144,43 +5190,43 @@
         <v>148</v>
       </c>
       <c r="C69" s="0" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="E69" s="0" t="n">
         <v>24</v>
       </c>
       <c r="F69" s="9"/>
       <c r="G69" s="5" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="I69" s="0" t="n">
         <v>24</v>
       </c>
       <c r="J69" s="11"/>
       <c r="K69" s="5" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="M69" s="0" t="n">
         <v>24</v>
       </c>
       <c r="O69" s="5" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="Q69" s="0" t="n">
         <v>24</v>
       </c>
       <c r="R69" s="11"/>
       <c r="S69" s="0" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="U69" s="0" t="n">
         <v>24</v>
       </c>
       <c r="W69" s="0" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="AB69" s="5" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5189,43 +5235,43 @@
       </c>
       <c r="B70" s="15"/>
       <c r="C70" s="0" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="E70" s="0" t="n">
         <v>25</v>
       </c>
       <c r="F70" s="9"/>
       <c r="G70" s="5" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="I70" s="0" t="n">
         <v>25</v>
       </c>
       <c r="J70" s="11"/>
       <c r="K70" s="0" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="M70" s="0" t="n">
         <v>25</v>
       </c>
       <c r="O70" s="0" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="Q70" s="0" t="n">
         <v>25</v>
       </c>
       <c r="R70" s="11"/>
       <c r="S70" s="0" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="U70" s="0" t="n">
         <v>25</v>
       </c>
       <c r="W70" s="0" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="AB70" s="5" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5234,7 +5280,7 @@
       </c>
       <c r="B71" s="15"/>
       <c r="C71" s="0" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="E71" s="0" t="n">
         <v>26</v>
@@ -5243,34 +5289,34 @@
         <v>126</v>
       </c>
       <c r="G71" s="5" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="I71" s="0" t="n">
         <v>26</v>
       </c>
       <c r="K71" s="5" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="M71" s="0" t="n">
         <v>26</v>
       </c>
       <c r="O71" s="0" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="Q71" s="0" t="n">
         <v>26</v>
       </c>
       <c r="S71" s="5" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="U71" s="0" t="n">
         <v>26</v>
       </c>
       <c r="W71" s="0" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="AB71" s="0" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5279,41 +5325,41 @@
       </c>
       <c r="B72" s="15"/>
       <c r="C72" s="5" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="E72" s="0" t="n">
         <v>27</v>
       </c>
       <c r="F72" s="10"/>
       <c r="G72" s="0" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="I72" s="0" t="n">
         <v>27</v>
       </c>
       <c r="K72" s="0" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="M72" s="0" t="n">
         <v>27</v>
       </c>
       <c r="O72" s="0" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="Q72" s="0" t="n">
         <v>27</v>
       </c>
       <c r="S72" s="0" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="U72" s="0" t="n">
         <v>27</v>
       </c>
       <c r="W72" s="0" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="AB72" s="5" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5321,41 +5367,41 @@
         <v>28</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="E73" s="0" t="n">
         <v>28</v>
       </c>
       <c r="F73" s="10"/>
       <c r="G73" s="0" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="I73" s="0" t="n">
         <v>28</v>
       </c>
       <c r="K73" s="0" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="M73" s="0" t="n">
         <v>28</v>
       </c>
       <c r="O73" s="0" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="Q73" s="0" t="n">
         <v>28</v>
       </c>
       <c r="S73" s="0" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="U73" s="0" t="n">
         <v>28</v>
       </c>
       <c r="W73" s="0" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="AB73" s="0" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5363,7 +5409,7 @@
         <v>29</v>
       </c>
       <c r="C74" s="0" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="E74" s="0" t="n">
         <v>29</v>
@@ -5372,13 +5418,13 @@
         <v>148</v>
       </c>
       <c r="G74" s="5" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="I74" s="0" t="n">
         <v>29</v>
       </c>
       <c r="K74" s="0" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="M74" s="0" t="n">
         <v>29</v>
@@ -5390,16 +5436,16 @@
         <v>29</v>
       </c>
       <c r="S74" s="0" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="U74" s="0" t="n">
         <v>29</v>
       </c>
       <c r="W74" s="0" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="AB74" s="0" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5407,20 +5453,20 @@
         <v>30</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="E75" s="0" t="n">
         <v>30</v>
       </c>
       <c r="F75" s="11"/>
       <c r="G75" s="0" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="I75" s="0" t="n">
         <v>30</v>
       </c>
       <c r="K75" s="0" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="M75" s="0" t="n">
         <v>30</v>
@@ -5432,237 +5478,237 @@
         <v>30</v>
       </c>
       <c r="S75" s="0" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="U75" s="0" t="n">
         <v>30</v>
       </c>
       <c r="W75" s="0" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="AB75" s="5" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB76" s="0" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB77" s="5" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB78" s="0" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB79" s="0" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB80" s="0" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H81" s="13"/>
+      <c r="H81" s="14"/>
       <c r="AB81" s="0" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB82" s="0" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB83" s="5" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB84" s="5" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB85" s="5" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB86" s="0" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB87" s="5" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB88" s="5" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB89" s="5" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB90" s="5" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB91" s="5" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB92" s="5" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB93" s="5" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB94" s="5" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB95" s="0" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB96" s="0" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB97" s="5" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB98" s="5" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB99" s="5" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB100" s="5" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB101" s="5" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB102" s="5" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB103" s="5" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB104" s="5" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB105" s="0" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB106" s="0" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB107" s="0" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB108" s="0" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB109" s="0" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB110" s="0" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB111" s="0" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB112" s="0" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB113" s="0" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB114" s="0" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB115" s="0" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB116" s="0" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB117" s="5" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB118" s="0" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AB119" s="0" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
     </row>
   </sheetData>
@@ -5727,115 +5773,115 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5897,233 +5943,233 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="B1" s="1"/>
       <c r="D1" s="1" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="19"/>
       <c r="G1" s="1" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="H1" s="1"/>
       <c r="J1" s="1" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="K1" s="1"/>
       <c r="L1" s="19"/>
       <c r="M1" s="1" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="N1" s="1"/>
       <c r="P1" s="1" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="Q1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="D2" s="0" t="s">
         <v>177</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>192</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>530</v>
-      </c>
-      <c r="J2" s="0" t="s">
-        <v>212</v>
+        <v>533</v>
+      </c>
+      <c r="J2" s="20" t="s">
+        <v>213</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="P2" s="5" t="s">
         <v>188</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="BG2" s="0"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="D3" s="0" t="s">
         <v>184</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="M3" s="0" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N3" s="0" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="P3" s="5" t="s">
         <v>195</v>
       </c>
       <c r="Q3" s="0" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="BG3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="0" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="D4" s="0" t="s">
         <v>191</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="M4" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="N4" s="0" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Q4" s="0" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="BG4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="0" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="K5" s="0" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="M5" s="0" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="N5" s="0" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="P5" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Q5" s="0" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="BG5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="0" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="K6" s="0" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="M6" s="0" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="N6" s="0" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="P6" s="0" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="Q6" s="0" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="BG6" s="0"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="0" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="P7" s="0" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="BG7" s="0"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="0" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="P8" s="0" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="BG8" s="0"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="0" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="BG9" s="0"/>
     </row>
@@ -6162,228 +6208,230 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B21" s="1"/>
       <c r="D21" s="1" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="19"/>
       <c r="G21" s="1" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="H21" s="1"/>
       <c r="J21" s="1" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="K21" s="1"/>
       <c r="L21" s="19"/>
       <c r="M21" s="1" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="N21" s="1"/>
       <c r="P21" s="1" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="Q21" s="1"/>
       <c r="BG21" s="0"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="N22" s="5" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="P22" s="5" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="Q22" s="5" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="BG22" s="0"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>576</v>
-      </c>
-      <c r="D23" s="0" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="J23" s="0" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="K23" s="0" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="M23" s="0" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="N23" s="0" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="P23" s="0" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="Q23" s="0" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="BG23" s="0"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
+        <v>449</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>585</v>
+      </c>
+      <c r="E24" s="0" t="s">
+        <v>586</v>
+      </c>
+      <c r="G24" s="0" t="s">
+        <v>438</v>
+      </c>
+      <c r="H24" s="0" t="s">
+        <v>587</v>
+      </c>
+      <c r="J24" s="0" t="s">
+        <v>425</v>
+      </c>
+      <c r="K24" s="0" t="s">
+        <v>588</v>
+      </c>
+      <c r="M24" s="0" t="s">
+        <v>440</v>
+      </c>
+      <c r="N24" s="0" t="s">
+        <v>589</v>
+      </c>
+      <c r="P24" s="0" t="s">
+        <v>406</v>
+      </c>
+      <c r="Q24" s="0" t="s">
+        <v>590</v>
+      </c>
+      <c r="BG24" s="0"/>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="s">
+        <v>591</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>592</v>
+      </c>
+      <c r="E25" s="0" t="s">
+        <v>593</v>
+      </c>
+      <c r="G25" s="0" t="s">
+        <v>445</v>
+      </c>
+      <c r="H25" s="0" t="s">
+        <v>594</v>
+      </c>
+      <c r="J25" s="0" t="s">
+        <v>432</v>
+      </c>
+      <c r="K25" s="0" t="s">
+        <v>595</v>
+      </c>
+      <c r="M25" s="0" t="s">
         <v>446</v>
       </c>
-      <c r="B24" s="0" t="s">
-        <v>583</v>
-      </c>
-      <c r="E24" s="0" t="s">
-        <v>584</v>
-      </c>
-      <c r="G24" s="0" t="s">
-        <v>435</v>
-      </c>
-      <c r="H24" s="0" t="s">
-        <v>585</v>
-      </c>
-      <c r="J24" s="0" t="s">
-        <v>422</v>
-      </c>
-      <c r="K24" s="0" t="s">
-        <v>586</v>
-      </c>
-      <c r="M24" s="0" t="s">
-        <v>437</v>
-      </c>
-      <c r="N24" s="0" t="s">
-        <v>587</v>
-      </c>
-      <c r="P24" s="0" t="s">
-        <v>403</v>
-      </c>
-      <c r="Q24" s="0" t="s">
-        <v>588</v>
-      </c>
-      <c r="BG24" s="0"/>
-    </row>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
-        <v>589</v>
-      </c>
-      <c r="B25" s="0" t="s">
-        <v>590</v>
-      </c>
-      <c r="E25" s="0" t="s">
-        <v>591</v>
-      </c>
-      <c r="G25" s="0" t="s">
-        <v>442</v>
-      </c>
-      <c r="H25" s="0" t="s">
-        <v>592</v>
-      </c>
-      <c r="J25" s="0" t="s">
-        <v>429</v>
-      </c>
-      <c r="K25" s="0" t="s">
-        <v>593</v>
-      </c>
-      <c r="M25" s="0" t="s">
-        <v>443</v>
-      </c>
       <c r="N25" s="0" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="P25" s="0" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="BG25" s="0"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
-        <v>595</v>
+      <c r="A26" s="20" t="s">
+        <v>597</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="J26" s="0" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="K26" s="0" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="M26" s="0" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="N26" s="0" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="P26" s="0" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="Q26" s="0" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="BG26" s="0"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D27" s="5"/>
       <c r="G27" s="5"/>
-      <c r="J27" s="5"/>
+      <c r="J27" s="0" t="s">
+        <v>603</v>
+      </c>
       <c r="M27" s="5"/>
       <c r="P27" s="0" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="BG27" s="0"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G28" s="5"/>
+      <c r="J28" s="0" t="s">
+        <v>604</v>
+      </c>
       <c r="M28" s="5"/>
       <c r="P28" s="0" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="BG28" s="0"/>
     </row>
@@ -6391,7 +6439,7 @@
       <c r="G29" s="20"/>
       <c r="M29" s="5"/>
       <c r="P29" s="0" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="BG29" s="0"/>
     </row>
@@ -6399,14 +6447,14 @@
       <c r="G30" s="20"/>
       <c r="M30" s="5"/>
       <c r="P30" s="0" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="BG30" s="0"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G31" s="20"/>
       <c r="P31" s="0" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="BG31" s="0"/>
     </row>
@@ -6429,7 +6477,7 @@
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="BG35" s="0"/>
       <c r="BH35" s="0"/>
@@ -6441,7 +6489,7 @@
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="BG36" s="0"/>
       <c r="BH36" s="0"/>
@@ -6453,13 +6501,13 @@
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E37" s="0" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="F37" s="0" t="n">
         <v>1.01</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="BG37" s="0"/>
       <c r="BH37" s="0"/>
@@ -6474,7 +6522,7 @@
         <v>1.02</v>
       </c>
       <c r="G38" s="0" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="BG38" s="0"/>
       <c r="BH38" s="0"/>
@@ -6489,7 +6537,7 @@
         <v>1.03</v>
       </c>
       <c r="G39" s="0" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="BG39" s="0"/>
       <c r="BH39" s="0"/>
@@ -6504,7 +6552,7 @@
         <v>1.04</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="BG40" s="0"/>
       <c r="BH40" s="0"/>
@@ -6519,7 +6567,7 @@
         <v>1.05</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="BG41" s="0"/>
       <c r="BH41" s="0"/>
@@ -6534,7 +6582,7 @@
         <v>1.06</v>
       </c>
       <c r="G42" s="0" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="BG42" s="0"/>
       <c r="BH42" s="0"/>
@@ -6549,7 +6597,7 @@
         <v>1.07</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="BG43" s="0"/>
       <c r="BH43" s="0"/>
@@ -6564,7 +6612,7 @@
         <v>1.08</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="BG44" s="0"/>
       <c r="BH44" s="0"/>
@@ -6579,7 +6627,7 @@
         <v>1.09</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="BG45" s="0"/>
       <c r="BH45" s="0"/>
@@ -6594,7 +6642,7 @@
         <v>1.1</v>
       </c>
       <c r="G46" s="0" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="BG46" s="0"/>
       <c r="BH46" s="0"/>
@@ -6609,7 +6657,7 @@
         <v>1.11</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="BG47" s="0"/>
       <c r="BH47" s="0"/>
@@ -6624,7 +6672,7 @@
         <v>1.12</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="BG48" s="0"/>
       <c r="BH48" s="0"/>
@@ -6716,6 +6764,12 @@
       <c r="BM57" s="0"/>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F58" s="0" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="G58" s="0" t="s">
+        <v>571</v>
+      </c>
       <c r="BG58" s="0"/>
       <c r="BH58" s="0"/>
       <c r="BI58" s="0"/>
@@ -6725,6 +6779,12 @@
       <c r="BM58" s="0"/>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F59" s="0" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G59" s="0" t="s">
+        <v>514</v>
+      </c>
       <c r="BG59" s="0"/>
       <c r="BH59" s="0"/>
       <c r="BI59" s="0"/>
@@ -6734,6 +6794,12 @@
       <c r="BM59" s="0"/>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F60" s="0" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G60" s="0" t="s">
+        <v>608</v>
+      </c>
       <c r="BG60" s="0"/>
       <c r="BH60" s="0"/>
       <c r="BI60" s="0"/>
@@ -6743,6 +6809,12 @@
       <c r="BM60" s="0"/>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F61" s="0" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G61" s="0" t="s">
+        <v>609</v>
+      </c>
       <c r="BG61" s="0"/>
       <c r="BH61" s="0"/>
       <c r="BI61" s="0"/>
@@ -6752,6 +6824,12 @@
       <c r="BM61" s="0"/>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F62" s="0" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="G62" s="0" t="s">
+        <v>522</v>
+      </c>
       <c r="BG62" s="0"/>
       <c r="BH62" s="0"/>
       <c r="BI62" s="0"/>
@@ -6761,6 +6839,12 @@
       <c r="BM62" s="0"/>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F63" s="0" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="G63" s="0" t="s">
+        <v>610</v>
+      </c>
       <c r="BG63" s="0"/>
       <c r="BH63" s="0"/>
       <c r="BI63" s="0"/>
@@ -6770,6 +6854,12 @@
       <c r="BM63" s="0"/>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F64" s="0" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G64" s="0" t="s">
+        <v>506</v>
+      </c>
       <c r="BG64" s="0"/>
       <c r="BH64" s="0"/>
       <c r="BI64" s="0"/>
@@ -6779,6 +6869,12 @@
       <c r="BM64" s="0"/>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F65" s="0" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="G65" s="0" t="s">
+        <v>524</v>
+      </c>
       <c r="BG65" s="0"/>
       <c r="BH65" s="0"/>
       <c r="BI65" s="0"/>
@@ -6788,6 +6884,12 @@
       <c r="BM65" s="0"/>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F66" s="0" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="G66" s="0" t="s">
+        <v>522</v>
+      </c>
       <c r="BG66" s="0"/>
       <c r="BH66" s="0"/>
       <c r="BI66" s="0"/>
@@ -6797,6 +6899,12 @@
       <c r="BM66" s="0"/>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F67" s="21" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G67" s="0" t="s">
+        <v>611</v>
+      </c>
       <c r="BG67" s="0"/>
       <c r="BH67" s="0"/>
       <c r="BI67" s="0"/>
@@ -6806,6 +6914,12 @@
       <c r="BM67" s="0"/>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F68" s="0" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="G68" s="0" t="s">
+        <v>506</v>
+      </c>
       <c r="BG68" s="0"/>
       <c r="BH68" s="0"/>
       <c r="BI68" s="0"/>
@@ -6815,6 +6929,12 @@
       <c r="BM68" s="0"/>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F69" s="0" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="G69" s="0" t="s">
+        <v>522</v>
+      </c>
       <c r="BG69" s="0"/>
       <c r="BH69" s="0"/>
       <c r="BI69" s="0"/>
@@ -6824,6 +6944,12 @@
       <c r="BM69" s="0"/>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F70" s="0" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="G70" s="0" t="s">
+        <v>571</v>
+      </c>
       <c r="BG70" s="0"/>
       <c r="BH70" s="0"/>
       <c r="BI70" s="0"/>
@@ -6833,6 +6959,12 @@
       <c r="BM70" s="0"/>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F71" s="0" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="G71" s="0" t="s">
+        <v>514</v>
+      </c>
       <c r="BG71" s="0"/>
       <c r="BH71" s="0"/>
       <c r="BI71" s="0"/>
@@ -6842,6 +6974,12 @@
       <c r="BM71" s="0"/>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F72" s="0" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="G72" s="0" t="s">
+        <v>608</v>
+      </c>
       <c r="BG72" s="0"/>
       <c r="BH72" s="0"/>
       <c r="BI72" s="0"/>
@@ -6851,6 +6989,12 @@
       <c r="BM72" s="0"/>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F73" s="0" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="G73" s="0" t="s">
+        <v>609</v>
+      </c>
       <c r="BG73" s="0"/>
       <c r="BH73" s="0"/>
       <c r="BI73" s="0"/>
@@ -6860,6 +7004,12 @@
       <c r="BM73" s="0"/>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F74" s="0" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="G74" s="0" t="s">
+        <v>610</v>
+      </c>
       <c r="BG74" s="0"/>
       <c r="BH74" s="0"/>
       <c r="BI74" s="0"/>
@@ -6869,6 +7019,12 @@
       <c r="BM74" s="0"/>
     </row>
     <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F75" s="0" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="G75" s="0" t="s">
+        <v>610</v>
+      </c>
       <c r="BG75" s="0"/>
       <c r="BH75" s="0"/>
       <c r="BI75" s="0"/>
@@ -6878,6 +7034,12 @@
       <c r="BM75" s="0"/>
     </row>
     <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F76" s="0" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="G76" s="0" t="s">
+        <v>571</v>
+      </c>
       <c r="BG76" s="0"/>
       <c r="BH76" s="0"/>
       <c r="BI76" s="0"/>
@@ -6887,6 +7049,12 @@
       <c r="BM76" s="0"/>
     </row>
     <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F77" s="0" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="G77" s="0" t="s">
+        <v>524</v>
+      </c>
       <c r="BG77" s="0"/>
       <c r="BH77" s="0"/>
       <c r="BI77" s="0"/>
@@ -6896,6 +7064,12 @@
       <c r="BM77" s="0"/>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F78" s="0" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="G78" s="0" t="s">
+        <v>571</v>
+      </c>
       <c r="BG78" s="0"/>
       <c r="BH78" s="0"/>
       <c r="BI78" s="0"/>
@@ -6905,6 +7079,12 @@
       <c r="BM78" s="0"/>
     </row>
     <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F79" s="21" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G79" s="0" t="s">
+        <v>611</v>
+      </c>
       <c r="BG79" s="0"/>
       <c r="BH79" s="0"/>
       <c r="BI79" s="0"/>
@@ -6914,6 +7094,12 @@
       <c r="BM79" s="0"/>
     </row>
     <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F80" s="0" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="G80" s="0" t="s">
+        <v>571</v>
+      </c>
       <c r="BG80" s="0"/>
       <c r="BH80" s="0"/>
       <c r="BI80" s="0"/>
@@ -6923,6 +7109,12 @@
       <c r="BM80" s="0"/>
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F81" s="0" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="G81" s="0" t="s">
+        <v>571</v>
+      </c>
       <c r="BG81" s="0"/>
       <c r="BH81" s="0"/>
       <c r="BI81" s="0"/>
@@ -6932,6 +7124,12 @@
       <c r="BM81" s="0"/>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F82" s="0" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="G82" s="0" t="s">
+        <v>514</v>
+      </c>
       <c r="BG82" s="0"/>
       <c r="BH82" s="0"/>
       <c r="BI82" s="0"/>
@@ -6941,6 +7139,12 @@
       <c r="BM82" s="0"/>
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F83" s="0" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="G83" s="0" t="s">
+        <v>608</v>
+      </c>
       <c r="BG83" s="0"/>
       <c r="BH83" s="0"/>
       <c r="BI83" s="0"/>
@@ -6950,6 +7154,12 @@
       <c r="BM83" s="0"/>
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F84" s="0" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="G84" s="0" t="s">
+        <v>609</v>
+      </c>
       <c r="BG84" s="0"/>
       <c r="BH84" s="0"/>
       <c r="BI84" s="0"/>
@@ -6959,6 +7169,12 @@
       <c r="BM84" s="0"/>
     </row>
     <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F85" s="0" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="G85" s="0" t="s">
+        <v>571</v>
+      </c>
       <c r="BG85" s="0"/>
       <c r="BH85" s="0"/>
       <c r="BI85" s="0"/>
@@ -6968,6 +7184,12 @@
       <c r="BM85" s="0"/>
     </row>
     <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F86" s="0" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="G86" s="0" t="s">
+        <v>522</v>
+      </c>
       <c r="BG86" s="0"/>
       <c r="BH86" s="0"/>
       <c r="BI86" s="0"/>
@@ -6977,6 +7199,12 @@
       <c r="BM86" s="0"/>
     </row>
     <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F87" s="0" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="G87" s="0" t="s">
+        <v>520</v>
+      </c>
       <c r="BG87" s="0"/>
       <c r="BH87" s="0"/>
       <c r="BI87" s="0"/>
@@ -6986,6 +7214,12 @@
       <c r="BM87" s="0"/>
     </row>
     <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F88" s="0" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="G88" s="0" t="s">
+        <v>524</v>
+      </c>
       <c r="BG88" s="0"/>
       <c r="BH88" s="0"/>
       <c r="BI88" s="0"/>
@@ -6995,6 +7229,12 @@
       <c r="BM88" s="0"/>
     </row>
     <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F89" s="0" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="G89" s="0" t="s">
+        <v>520</v>
+      </c>
       <c r="BG89" s="0"/>
       <c r="BH89" s="0"/>
       <c r="BI89" s="0"/>
@@ -7004,6 +7244,12 @@
       <c r="BM89" s="0"/>
     </row>
     <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F90" s="0" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="G90" s="0" t="s">
+        <v>611</v>
+      </c>
       <c r="BG90" s="0"/>
       <c r="BH90" s="0"/>
       <c r="BI90" s="0"/>
@@ -7013,6 +7259,12 @@
       <c r="BM90" s="0"/>
     </row>
     <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F91" s="21" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G91" s="0" t="s">
+        <v>571</v>
+      </c>
       <c r="BG91" s="0"/>
       <c r="BH91" s="0"/>
       <c r="BI91" s="0"/>
@@ -7022,6 +7274,12 @@
       <c r="BM91" s="0"/>
     </row>
     <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F92" s="0" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="G92" s="0" t="s">
+        <v>520</v>
+      </c>
       <c r="BG92" s="0"/>
       <c r="BH92" s="0"/>
       <c r="BI92" s="0"/>
@@ -7031,6 +7289,12 @@
       <c r="BM92" s="0"/>
     </row>
     <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F93" s="0" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="G93" s="0" t="s">
+        <v>571</v>
+      </c>
       <c r="BG93" s="0"/>
       <c r="BH93" s="0"/>
       <c r="BI93" s="0"/>
@@ -7040,6 +7304,12 @@
       <c r="BM93" s="0"/>
     </row>
     <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F94" s="0" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="G94" s="0" t="s">
+        <v>514</v>
+      </c>
       <c r="BG94" s="0"/>
       <c r="BH94" s="0"/>
       <c r="BI94" s="0"/>
@@ -7049,6 +7319,12 @@
       <c r="BM94" s="0"/>
     </row>
     <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F95" s="0" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="G95" s="0" t="s">
+        <v>608</v>
+      </c>
       <c r="BG95" s="0"/>
       <c r="BH95" s="0"/>
       <c r="BI95" s="0"/>
@@ -7058,6 +7334,12 @@
       <c r="BM95" s="0"/>
     </row>
     <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F96" s="0" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="G96" s="0" t="s">
+        <v>609</v>
+      </c>
       <c r="BG96" s="0"/>
       <c r="BH96" s="0"/>
       <c r="BI96" s="0"/>
@@ -7067,6 +7349,12 @@
       <c r="BM96" s="0"/>
     </row>
     <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F97" s="0" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="G97" s="0" t="s">
+        <v>520</v>
+      </c>
       <c r="BG97" s="0"/>
       <c r="BH97" s="0"/>
       <c r="BI97" s="0"/>
@@ -7076,6 +7364,12 @@
       <c r="BM97" s="0"/>
     </row>
     <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F98" s="0" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="G98" s="0" t="s">
+        <v>522</v>
+      </c>
       <c r="BG98" s="0"/>
       <c r="BH98" s="0"/>
       <c r="BI98" s="0"/>
@@ -7085,6 +7379,12 @@
       <c r="BM98" s="0"/>
     </row>
     <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F99" s="0" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="G99" s="0" t="s">
+        <v>522</v>
+      </c>
       <c r="BG99" s="0"/>
       <c r="BH99" s="0"/>
       <c r="BI99" s="0"/>
@@ -7094,6 +7394,12 @@
       <c r="BM99" s="0"/>
     </row>
     <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F100" s="0" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="G100" s="0" t="s">
+        <v>524</v>
+      </c>
       <c r="BG100" s="0"/>
       <c r="BH100" s="0"/>
       <c r="BI100" s="0"/>
@@ -7103,6 +7409,12 @@
       <c r="BM100" s="0"/>
     </row>
     <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F101" s="0" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="G101" s="0" t="s">
+        <v>611</v>
+      </c>
       <c r="BG101" s="0"/>
       <c r="BH101" s="0"/>
       <c r="BI101" s="0"/>
@@ -7112,6 +7424,12 @@
       <c r="BM101" s="0"/>
     </row>
     <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F102" s="0" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="G102" s="0" t="s">
+        <v>520</v>
+      </c>
       <c r="BG102" s="0"/>
       <c r="BH102" s="0"/>
       <c r="BI102" s="0"/>
@@ -7121,6 +7439,12 @@
       <c r="BM102" s="0"/>
     </row>
     <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F103" s="21" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G103" s="0" t="s">
+        <v>571</v>
+      </c>
       <c r="BG103" s="0"/>
       <c r="BH103" s="0"/>
       <c r="BI103" s="0"/>
@@ -7130,6 +7454,12 @@
       <c r="BM103" s="0"/>
     </row>
     <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F104" s="0" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="G104" s="0" t="s">
+        <v>514</v>
+      </c>
       <c r="BG104" s="0"/>
       <c r="BH104" s="0"/>
       <c r="BI104" s="0"/>
@@ -7139,6 +7469,12 @@
       <c r="BM104" s="0"/>
     </row>
     <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F105" s="0" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="G105" s="0" t="s">
+        <v>608</v>
+      </c>
       <c r="BG105" s="0"/>
       <c r="BH105" s="0"/>
       <c r="BI105" s="0"/>
@@ -7148,6 +7484,12 @@
       <c r="BM105" s="0"/>
     </row>
     <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F106" s="0" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="G106" s="0" t="s">
+        <v>609</v>
+      </c>
       <c r="BG106" s="0"/>
       <c r="BH106" s="0"/>
       <c r="BI106" s="0"/>
@@ -7157,6 +7499,12 @@
       <c r="BM106" s="0"/>
     </row>
     <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F107" s="0" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="G107" s="0" t="s">
+        <v>611</v>
+      </c>
       <c r="BG107" s="0"/>
       <c r="BH107" s="0"/>
       <c r="BI107" s="0"/>
@@ -7166,6 +7514,12 @@
       <c r="BM107" s="0"/>
     </row>
     <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F108" s="0" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="G108" s="0" t="s">
+        <v>520</v>
+      </c>
       <c r="BG108" s="0"/>
       <c r="BH108" s="0"/>
       <c r="BI108" s="0"/>
@@ -7175,6 +7529,12 @@
       <c r="BM108" s="0"/>
     </row>
     <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F109" s="0" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="G109" s="0" t="s">
+        <v>608</v>
+      </c>
       <c r="BG109" s="0"/>
       <c r="BH109" s="0"/>
       <c r="BI109" s="0"/>
@@ -7184,6 +7544,12 @@
       <c r="BM109" s="0"/>
     </row>
     <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F110" s="0" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="G110" s="0" t="s">
+        <v>608</v>
+      </c>
       <c r="BG110" s="0"/>
       <c r="BH110" s="0"/>
       <c r="BI110" s="0"/>
@@ -7229,6 +7595,7 @@
       <c r="BM114" s="0"/>
     </row>
     <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F115" s="21"/>
       <c r="BG115" s="0"/>
       <c r="BH115" s="0"/>
       <c r="BI115" s="0"/>
@@ -8304,68 +8671,68 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="23" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="25"/>
       <c r="B2" s="26" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="25"/>
       <c r="B3" s="26" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="25" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="25"/>
       <c r="B5" s="26" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="25"/>
       <c r="B6" s="26" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="27"/>
       <c r="B7" s="28" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25"/>
       <c r="B10" s="26" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27"/>
       <c r="B11" s="28" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8374,42 +8741,42 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="23" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="25"/>
       <c r="B14" s="26" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="25"/>
       <c r="B15" s="26" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27"/>
       <c r="B16" s="28" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="27"/>
       <c r="B19" s="28" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8418,22 +8785,22 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="B21" s="24" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="25"/>
       <c r="B22" s="26" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="25"/>
       <c r="B23" s="26" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8442,10 +8809,10 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8458,7 +8825,7 @@
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="27"/>
       <c r="B27" s="28" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8467,15 +8834,15 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="27" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="B29" s="28" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="23" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="B31" s="29" t="n">
         <v>1.12</v>
@@ -8487,7 +8854,7 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="25" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="B33" s="30" t="s">
         <v>90</v>
@@ -8496,27 +8863,27 @@
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="27"/>
       <c r="B34" s="28" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="23" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="B36" s="29" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="25"/>
       <c r="B37" s="30" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="25"/>
       <c r="B38" s="30" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8525,18 +8892,18 @@
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="27" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="B40" s="28" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="23" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B43" s="24" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="E43" s="0"/>
       <c r="F43" s="0"/>
@@ -8544,7 +8911,7 @@
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="25"/>
       <c r="B44" s="26" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="E44" s="0"/>
       <c r="F44" s="0"/>
@@ -8557,10 +8924,10 @@
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="27" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="B46" s="28" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="E46" s="0"/>
       <c r="F46" s="0"/>
@@ -8571,23 +8938,23 @@
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="23" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="B48" s="24" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="F48" s="0"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="25"/>
       <c r="B49" s="26" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="25"/>
       <c r="B50" s="26" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8598,10 +8965,10 @@
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="27" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="B52" s="28" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="D52" s="0"/>
       <c r="E52" s="0"/>
@@ -8615,10 +8982,10 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="23" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="B54" s="24" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="D54" s="0"/>
       <c r="E54" s="0"/>
@@ -8633,7 +9000,7 @@
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="27" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="B56" s="28" t="s">
         <v>121</v>
@@ -8835,7 +9202,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="33" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="B1" s="33"/>
     </row>

</xml_diff>